<commit_message>
Code bereinigt und Dateien gelöscht
</commit_message>
<xml_diff>
--- a/charts/Burndown-Chart.xlsx
+++ b/charts/Burndown-Chart.xlsx
@@ -1,25 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29415"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Siepmann\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\s-pon\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE34B8E9-AA30-426A-B1B4-1D2400251309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6D13FE3-B097-4281-A371-F166A1BD5290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -62,23 +59,23 @@
     <t>Gesamtaufwand</t>
   </si>
   <si>
+    <t>Restaufwand:</t>
+  </si>
+  <si>
     <t>Wochenaufwand:</t>
   </si>
   <si>
-    <t>ab Kalenderwoche 43 werden in dieser Spalte jede Woche die geleisteten Stunden (Aufwand) der vergangenen Woche eingetragen</t>
+    <t>In dieser Spalte wird jede Woche der neu geschätzte Restaufwand eingetragen ( siehe Folie "Aktuell geschätzter Restaufwand" aus Vorlesung "KW42" )</t>
   </si>
   <si>
-    <t>Restaufwand:</t>
-  </si>
-  <si>
-    <t>In dieser Spalte wird jede Woche der neu geschätzte Restaufwand eingetragen ( siehe Folie "Aktuell geschätzter Restaufwand" aus Vorlesung "KW42" )</t>
+    <t>ab Kalenderwoche 43 werden in dieser Spalte jede Woche die geleisteten Stunden (Aufwand) der vergangenen Woche eingetragen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -164,8 +161,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Explanatory Text" xfId="1" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Erklärender Text" xfId="1" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -251,7 +248,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -331,10 +328,10 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Tabelle1!$A$5:$A$20</c:f>
+              <c:f>Tabelle1!$A$5:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>43</c:v>
                 </c:pt>
@@ -370,21 +367,51 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tabelle1!$B$5:$B$20</c:f>
+              <c:f>Tabelle1!$B$5:$B$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>30</c:v>
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>56</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -450,10 +477,10 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Tabelle1!$A$5:$A$20</c:f>
+              <c:f>Tabelle1!$A$5:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>43</c:v>
                 </c:pt>
@@ -489,66 +516,51 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tabelle1!$C$5:$C$20</c:f>
+              <c:f>Tabelle1!$C$5:$C$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>570</c:v>
+                  <c:v>473</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>570</c:v>
+                  <c:v>440</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>570</c:v>
+                  <c:v>403</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>570</c:v>
+                  <c:v>365</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>570</c:v>
+                  <c:v>321</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>570</c:v>
+                  <c:v>301</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>570</c:v>
+                  <c:v>268</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>570</c:v>
+                  <c:v>220</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>570</c:v>
+                  <c:v>148</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>570</c:v>
+                  <c:v>134</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>570</c:v>
+                  <c:v>129</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>570</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>570</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>570</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>570</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>570</c:v>
+                  <c:v>73</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -608,10 +620,10 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Tabelle1!$A$5:$A$20</c:f>
+              <c:f>Tabelle1!$A$5:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>43</c:v>
                 </c:pt>
@@ -647,66 +659,51 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tabelle1!$D$5:$D$20</c:f>
+              <c:f>Tabelle1!$D$5:$D$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>30</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>30</c:v>
+                  <c:v>64</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>30</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>30</c:v>
+                  <c:v>139</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>30</c:v>
+                  <c:v>183</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>30</c:v>
+                  <c:v>203</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>30</c:v>
+                  <c:v>236</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>30</c:v>
+                  <c:v>284</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>30</c:v>
+                  <c:v>356</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>30</c:v>
+                  <c:v>370</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>30</c:v>
+                  <c:v>375</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>30</c:v>
+                  <c:v>431</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -766,10 +763,10 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Tabelle1!$A$5:$A$20</c:f>
+              <c:f>Tabelle1!$A$5:$A$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>43</c:v>
                 </c:pt>
@@ -805,66 +802,51 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tabelle1!$E$5:$E$20</c:f>
+              <c:f>Tabelle1!$E$5:$E$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>600</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>600</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>600</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>600</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>600</c:v>
+                  <c:v>504</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1109,9 +1091,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1149,7 +1131,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1255,7 +1237,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1397,7 +1379,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1406,7 +1388,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:E46"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" style="1" customWidth="1"/>
@@ -1416,7 +1398,7 @@
     <col min="6" max="1025" width="11.42578125"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="12.6">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1424,7 +1406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="12.6">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1432,7 +1414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="12.75">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1449,318 +1431,302 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="12.75">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>43</v>
       </c>
       <c r="B5" s="3">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" s="3">
-        <v>570</v>
+        <f>504-B5</f>
+        <v>473</v>
       </c>
       <c r="D5" s="4">
         <f>B5</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E5" s="5">
         <f>C5+D5</f>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
-        <f t="shared" ref="A6:A15" si="0">A5+1</f>
+        <f t="shared" ref="A6:A14" si="0">A5+1</f>
         <v>44</v>
       </c>
-      <c r="B6" s="3"/>
+      <c r="B6" s="3">
+        <v>33</v>
+      </c>
       <c r="C6" s="3">
-        <f t="shared" ref="C6:C20" si="1">C5</f>
-        <v>570</v>
+        <f>C5-B6</f>
+        <v>440</v>
       </c>
       <c r="D6" s="4">
-        <f>B6+D5</f>
-        <v>30</v>
+        <f t="shared" ref="D6:D20" si="1">B6+D5</f>
+        <v>64</v>
       </c>
       <c r="E6" s="5">
         <f t="shared" ref="E5:E20" si="2">C6+D6</f>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="B7" s="3"/>
+      <c r="B7" s="3">
+        <v>37</v>
+      </c>
       <c r="C7" s="3">
+        <f>C6-B7</f>
+        <v>403</v>
+      </c>
+      <c r="D7" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D7" s="4">
-        <f t="shared" ref="D6:D20" si="3">B7+D6</f>
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="E7" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="B8" s="3"/>
+      <c r="B8" s="3">
+        <v>38</v>
+      </c>
       <c r="C8" s="3">
+        <f>C7-B8</f>
+        <v>365</v>
+      </c>
+      <c r="D8" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D8" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <v>139</v>
       </c>
       <c r="E8" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="B9" s="3"/>
+      <c r="B9" s="3">
+        <v>44</v>
+      </c>
       <c r="C9" s="3">
+        <f>C8-B9</f>
+        <v>321</v>
+      </c>
+      <c r="D9" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D9" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <v>183</v>
       </c>
       <c r="E9" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="B10" s="3"/>
+      <c r="B10" s="3">
+        <v>20</v>
+      </c>
       <c r="C10" s="3">
+        <f>C9-B10</f>
+        <v>301</v>
+      </c>
+      <c r="D10" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D10" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <v>203</v>
       </c>
       <c r="E10" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="B11" s="3"/>
+      <c r="B11" s="3">
+        <v>33</v>
+      </c>
       <c r="C11" s="3">
+        <f>C10-B11</f>
+        <v>268</v>
+      </c>
+      <c r="D11" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D11" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <v>236</v>
       </c>
       <c r="E11" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="B12" s="3"/>
+      <c r="B12" s="3">
+        <v>48</v>
+      </c>
       <c r="C12" s="3">
+        <f>C11-B12</f>
+        <v>220</v>
+      </c>
+      <c r="D12" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D12" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <v>284</v>
       </c>
       <c r="E12" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="B13" s="3"/>
+      <c r="B13" s="3">
+        <v>72</v>
+      </c>
       <c r="C13" s="3">
+        <f>C12-B13</f>
+        <v>148</v>
+      </c>
+      <c r="D13" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D13" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <v>356</v>
       </c>
       <c r="E13" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="B14" s="3"/>
+      <c r="B14" s="3">
+        <v>14</v>
+      </c>
       <c r="C14" s="3">
+        <f>C13-B14</f>
+        <v>134</v>
+      </c>
+      <c r="D14" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D14" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <v>370</v>
       </c>
       <c r="E14" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>1</v>
       </c>
-      <c r="B15" s="3"/>
+      <c r="B15" s="3">
+        <v>5</v>
+      </c>
       <c r="C15" s="3">
+        <f>C14-B15</f>
+        <v>129</v>
+      </c>
+      <c r="D15" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D15" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <v>375</v>
       </c>
       <c r="E15" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="12.75">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <f>A15+1</f>
         <v>2</v>
       </c>
-      <c r="B16" s="3"/>
+      <c r="B16" s="3">
+        <v>56</v>
+      </c>
       <c r="C16" s="3">
+        <f>C15-B16</f>
+        <v>73</v>
+      </c>
+      <c r="D16" s="4">
         <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D16" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
+        <v>431</v>
       </c>
       <c r="E16" s="5">
         <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="12.75">
-      <c r="A17" s="4">
-        <f>A16+1</f>
-        <v>3</v>
-      </c>
+        <v>504</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="4"/>
       <c r="B17" s="3"/>
-      <c r="C17" s="3">
-        <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D17" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
-      </c>
-      <c r="E17" s="5">
-        <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="12.75">
+      <c r="C17" s="3"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="4"/>
       <c r="B18" s="3"/>
-      <c r="C18" s="3">
-        <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D18" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
-      </c>
-      <c r="E18" s="5">
-        <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="12.75">
+      <c r="C18" s="3"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="4"/>
       <c r="B19" s="3"/>
-      <c r="C19" s="3">
-        <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D19" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
-      </c>
-      <c r="E19" s="5">
-        <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="12.75">
+      <c r="C19" s="3"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="4"/>
       <c r="B20" s="3"/>
-      <c r="C20" s="3">
-        <f t="shared" si="1"/>
-        <v>570</v>
-      </c>
-      <c r="D20" s="4">
-        <f t="shared" si="3"/>
-        <v>30</v>
-      </c>
-      <c r="E20" s="5">
-        <f t="shared" si="2"/>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" ht="12.75">
+      <c r="C20" s="3"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="5"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:1" ht="12.75">
-      <c r="A43" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1">
-      <c r="A45" s="6" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1">
-      <c r="A46" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>